<commit_message>
fix: repair text mangled by the em-dash pass; rebuild xlsx with a Summary sheet
The first em-dash conversion nested its placeholders and corrupted 15 lines
where a quoted string sat inside a code span (aria-label, type="number",
alt=""). Reverted those seven files and reran a corrected pass that only
protects code spans and restores innermost-first. Scanned the whole corpus:
no sentinels or control characters remain.

xlsx regenerated from the current markdown so the two stay in sync, now with
the test summary as a second sheet per §14.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/checklist/gui-checklist.xlsx
+++ b/checklist/gui-checklist.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="GUI Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GUI Checklist'!$A$1:$I$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Checklist'!$A$1:$I$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,8 +32,15 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -41,26 +49,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="002F5597"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,23 +65,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -461,15 +441,15 @@
   <dimension ref="A1:I111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-    <col width="24" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="72" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,7 +470,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Checklist item</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -545,7 +525,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -584,7 +564,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -623,14 +603,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hiển thị "30,000,000 ₫" — có ký hiệu ₫ và phân cách hàng nghìn (dùng dấu phẩy thay vì dấu chấm, chấp nhận được vì `Number.toLocaleString()` mặc định en-US, không thuộc phạm vi item này)</t>
+          <t>Hiển thị "30,000,000 ₫": có ký hiệu ₫ và phân cách hàng nghìn (dùng dấu phẩy thay vì dấu chấm, chấp nhận được vì `Number.toLocaleString()` mặc định en-US, không thuộc phạm vi item này)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -662,14 +642,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Nút dùng `bg-green-600` (xanh lá), không phải xanh dương; đối chiếu ngay với nút "Thêm vào giỏ" cùng chức năng ở trang danh sách lại đúng là `bg-blue-600` — không nhất quán trong cùng hệ thống, vi phạm FR-21</t>
+          <t>Nút dùng `bg-green-600` (xanh lá), không phải xanh dương; đối chiếu ngay với nút "Thêm vào giỏ" cùng chức năng ở trang danh sách lại đúng là `bg-blue-600`, không nhất quán trong cùng hệ thống, vi phạm FR-21</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -709,14 +689,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Thiếu trường Danh mục trên cả 5/5 sản phẩm, dù backend đã có `category_id` cho mọi sản phẩm (xác nhận qua `GET /api/products`) — vi phạm trực tiếp FR-06</t>
+          <t>Thiếu trường Danh mục trên cả 5/5 sản phẩm, dù backend đã có `category_id` cho mọi sản phẩm (xác nhận qua `GET /api/products`), vi phạm trực tiếp FR-06</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -756,7 +736,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -787,7 +767,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Tên sản phẩm dài (&gt;60 ký tự) không làm vỡ layout — có xử lý truncate hoặc wrap hợp lý, không tràn ra ngoài khung</t>
+          <t>Tên sản phẩm dài (&gt;60 ký tự) không làm vỡ layout, có xử lý truncate hoặc wrap hợp lý, không tràn ra ngoài khung</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -795,14 +775,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Không có sản phẩm thật nào &gt;60 ký tự trong SUT (dài nhất ~24 ký tự); kiểm thử bằng cách tạm chèn chuỗi dài qua DOM vào `&lt;h1&gt;` thật của trang — `white-space: normal` mặc định, text wrap đúng, không tràn khung (`scrollWidth` = `clientWidth`)</t>
+          <t>Không có sản phẩm thật nào &gt;60 ký tự trong SUT (dài nhất ~24 ký tự); kiểm thử bằng cách tạm chèn chuỗi dài qua DOM vào `&lt;h1&gt;` thật của trang, `white-space: normal` mặc định, text wrap đúng, không tràn khung (`scrollWidth` = `clientWidth`)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -834,14 +814,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Cùng phương pháp GUI-007: chèn mô tả dài — không có `max-height`/`overflow: hidden`, text hiển thị đầy đủ, không bị cắt cụt</t>
+          <t>Cùng phương pháp GUI-007: chèn mô tả dài, không có `max-height`/`overflow: hidden`, text hiển thị đầy đủ, không bị cắt cụt</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -865,7 +845,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Font chữ, cỡ chữ, màu chữ nhất quán với các màn hình khác (Home, product grid) — không lệch style</t>
+          <t>Font chữ, cỡ chữ, màu chữ nhất quán với các màn hình khác (Home, product grid), không lệch style</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -873,7 +853,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -912,14 +892,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Đo bằng công thức WCAG relative luminance qua JS trên nền hiệu lực thật (trắng): tên (đen/trắng) ~21:1, giá (`text-red-600`/trắng) 4.83:1, mô tả (`text-gray-700`/trắng) 10.31:1 — cả 3 đều đạt chuẩn AA cho chữ thường</t>
+          <t>Đo bằng công thức WCAG relative luminance qua JS trên nền hiệu lực thật (trắng): tên (đen/trắng) ~21:1, giá (`text-red-600`/trắng) 4.83:1, mô tả (`text-gray-700`/trắng) 10.31:1, cả 3 đều đạt chuẩn AA cho chữ thường</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -943,7 +923,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Layout responsive hợp lý ở cả desktop và mobile — ảnh, thông tin, nút bấm không đè lên nhau khi thu nhỏ màn hình</t>
+          <t>Layout responsive hợp lý ở cả desktop và mobile, ảnh, thông tin, nút bấm không đè lên nhau khi thu nhỏ màn hình</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -951,14 +931,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử ở các độ rộng 1400px, 757px, 625px (625px là giới hạn nhỏ nhất công cụ resize cho phép trong môi trường này) — không phát hiện chồng lấn. Phát hiện thêm 1 class CSS đáng ngờ `.bug-mobile-hidden { @media(max-width:640px){margin-right:-100px} }` gắn trên chính nút "Thêm vào giỏ hàng", nhưng verify thực tế không gây lệch vị trí nút ở các độ rộng đã test (margin-right âm không dịch chuyển box vì nút là item cuối trong flex-column `self-start`) — không đủ bằng chứng để kết luận Failed, ghi nhận là rủi ro tiềm ẩn cần theo dõi ở màn hình thật &lt;625px</t>
+          <t>Kiểm thử ở các độ rộng 1400px, 757px, 625px (625px là giới hạn nhỏ nhất công cụ resize cho phép trong môi trường này), không phát hiện chồng lấn. Phát hiện thêm 1 class CSS đáng ngờ `.bug-mobile-hidden { @media(max-width:640px){margin-right:-100px} }` gắn trên chính nút "Thêm vào giỏ hàng", nhưng verify thực tế không gây lệch vị trí nút ở các độ rộng đã test (margin-right âm không dịch chuyển box vì nút là item cuối trong flex-column `self-start`), không đủ bằng chứng để kết luận Failed, ghi nhận là rủi ro tiềm ẩn cần theo dõi ở màn hình thật &lt;625px</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -990,14 +970,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra DOM: không có bất kỳ wrapper skeleton/placeholder nào quanh `&lt;img&gt;` — ảnh render thẳng, không có loading state nào quan sát được</t>
+          <t>Kiểm tra DOM: không có bất kỳ wrapper skeleton/placeholder nào quanh `&lt;img&gt;`, ảnh render thẳng, không có loading state nào quan sát được</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1037,14 +1017,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử thực tế: nhập 0 vào ô Số lượng rồi thêm vào giỏ — hệ thống chấp nhận, item xuất hiện trong giỏ với "Số lượng: 0", "Thành tiền: 0 ₫". Input không có `min`/`max`, source xác nhận không có validate nào (`onChange` chỉ set state trực tiếp)</t>
+          <t>Kiểm thử thực tế: nhập 0 vào ô Số lượng rồi thêm vào giỏ, hệ thống chấp nhận, item xuất hiện trong giỏ với "Số lượng: 0", "Thành tiền: 0 ₫". Ô nhập không khai báo `min`/`max`, và không có thông báo lỗi nào xuất hiện ở bất kỳ thời điểm nào (lúc gõ, lúc rời ô, lúc submit)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1084,7 +1064,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1123,7 +1103,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -1170,14 +1150,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Gõ "abc" vào ô `type="number"` — trình duyệt (Chromium) tự động từ chối, ô hiển thị rỗng, không cho nhập ký tự chữ</t>
+          <t>Gõ "abc" vào ô `type="number"`: trình duyệt (Chromium) tự động từ chối, ô hiển thị rỗng, không cho nhập ký tự chữ</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
@@ -1209,14 +1189,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Không có bất kỳ thông báo lỗi nào xuất hiện ở bất kỳ vị trí nào cho các giá trị 0/để trống — hệ thống hoặc im lặng bỏ qua hoặc (với 0) âm thầm chấp nhận, không bao giờ báo lỗi</t>
+          <t>Không có bất kỳ thông báo lỗi nào xuất hiện ở bất kỳ vị trí nào cho các giá trị 0/để trống, hệ thống hoặc im lặng bỏ qua hoặc (với 0) âm thầm chấp nhận, không bao giờ báo lỗi</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1256,7 +1236,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1292,17 +1272,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>AI (sửa bởi Human — xem Entry #2 ai-audit-report.md)</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
+          <t>AI (sửa bởi Human: xem Entry #2 ai-audit-report.md)</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Không có nút +/- nào trong DOM (chỉ có 1 ô input số) trên cả 5 sản phẩm — tính năng không tồn tại trong SUT nên không thể kiểm thử (theo quy ước N/A đã thống nhất ở Entry #2)</t>
+          <t>Không có nút +/- nào trong DOM (chỉ có 1 ô input số) trên cả 5 sản phẩm, tính năng không tồn tại trong SUT nên không thể kiểm thử (theo quy ước N/A đã thống nhất ở Entry #2)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -1334,14 +1314,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Nút không bao giờ bị disable ở bất kỳ trạng thái nào. Tệ hơn: hành vi quan sát được ngược lại — mỗi "lần thêm hợp lệ" luôn cần đúng 2 lần bấm liên tiếp (lần đầu luôn bị bỏ qua im lặng, xác nhận lặp lại trên nhiều sản phẩm) — xem BUG-IA04-PRODUCTDETAIL-001</t>
+          <t>Nút không bao giờ bị disable ở bất kỳ trạng thái nào. Tệ hơn: hành vi quan sát được ngược lại, mỗi "lần thêm hợp lệ" luôn cần đúng 2 lần bấm liên tiếp (lần đầu luôn bị bỏ qua im lặng, xác nhận lặp lại trên nhiều sản phẩm), xem BUG-IA04-PRODUCTDETAIL-001</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -1381,14 +1361,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Không quan sát được bất kỳ validate nào ở bất kỳ thời điểm (gõ, rời ô, submit) — thử cả 3 thời điểm với giá trị 0/âm/để trống, không lần nào xuất hiện lỗi</t>
+          <t>Không quan sát được bất kỳ validate nào ở bất kỳ thời điểm (gõ, rời ô, submit), thử cả 3 thời điểm với giá trị 0/âm/để trống, không lần nào xuất hiện lỗi</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1428,14 +1408,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Cơ chế enforcement của Chromium cho `type="number"` áp dụng như nhau cho gõ tay và dán (paste) — đã xác nhận hành vi gõ tay ở GUI-016 dùng chung engine input filtering</t>
+          <t>Cơ chế enforcement của Chromium cho `type="number"` áp dụng như nhau cho gõ tay và dán (paste), đã xác nhận hành vi gõ tay ở GUI-016 dùng chung engine input filtering</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
@@ -1467,14 +1447,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Không có breadcrumb nào trên trang, xác nhận qua DOM (`[class*="breadcrumb"]` = null) trên cả 5 sản phẩm — vi phạm FR-23 ("Breadcrumb bắt buộc có ở... Chi tiết sản phẩm")</t>
+          <t>Không có breadcrumb nào trên trang, xác nhận qua DOM (`[class*="breadcrumb"]` = null) trên cả 5 sản phẩm, vi phạm FR-23 ("Breadcrumb bắt buộc có ở... Chi tiết sản phẩm")</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -1514,14 +1494,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Không thể kiểm thử — breadcrumb không tồn tại (hệ quả trực tiếp của GUI-023)</t>
+          <t>Không thể kiểm thử: breadcrumb không tồn tại (hệ quả trực tiếp của GUI-023)</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1561,14 +1541,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Không thể kiểm thử — breadcrumb không tồn tại (hệ quả trực tiếp của GUI-023)</t>
+          <t>Không thể kiểm thử: breadcrumb không tồn tại (hệ quả trực tiếp của GUI-023)</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1608,14 +1588,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Không có nút/link "Quay lại" nào ngoài breadcrumb (vốn cũng không tồn tại) và logo "EShop" trên navbar — người dùng chỉ còn cách dùng nút Back trình duyệt</t>
+          <t>Không có nút/link "Quay lại" nào ngoài breadcrumb (vốn cũng không tồn tại) và logo "EShop" trên navbar, người dùng chỉ còn cách dùng nút Back trình duyệt</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -1655,17 +1635,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Nội dung danh sách hiển thị đúng nhưng vị trí cuộn bị reset về đầu trang sau khi Back, không giữ lại vị trí đã cuộn trước đó</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr"/>
+          <t>Trên bản localhost tải nhanh, vị trí cuộn được khôi phục đúng sau khi Back. Nhưng khi danh sách sản phẩm về chậm (mô phỏng mạng chậm, cùng kỹ thuật đã dùng ở GUI-079), trình duyệt khôi phục cuộn lúc trang còn rỗng nên bị kẹp về 0, và khi dữ liệu về thì vị trí cuộn không được khôi phục lại nữa: đo được scrollY = 0 ở mọi mốc thời gian sau khi lưới đã render đủ 5 sản phẩm. Đây là kịch bản người dùng thật gặp trên mạng chậm hoặc trang dài</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-027-scroll-lost-slow-load.png</t>
+        </is>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
           <t>BUG-IA03-PRODUCTDETAIL-002</t>
@@ -1698,7 +1682,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1737,14 +1721,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Navbar (Giỏ hàng/Đăng nhập/Đăng ký hoặc Giỏ hàng/Chào .../Thoát) không có bất kỳ cơ chế highlight active-link nào — do đó không có mục nào bị highlight sai (Passed theo đúng nghĩa đen của item; việc thiếu hoàn toàn active-state là một nhận xét khác, không thuộc phạm vi item này)</t>
+          <t>Navbar (Giỏ hàng/Đăng nhập/Đăng ký hoặc Giỏ hàng/Chào .../Thoát) không có bất kỳ cơ chế highlight active-link nào, do đó không có mục nào bị highlight sai (Passed theo đúng nghĩa đen của item; việc thiếu hoàn toàn active-state là một nhận xét khác, không thuộc phạm vi item này)</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
@@ -1768,7 +1752,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Nếu có phần "Sản phẩm liên quan" ở cuối trang, bấm vào một sản phẩm liên quan điều hướng đúng sang trang chi tiết của sản phẩm đó (xác nhận tính năng tồn tại trước khi Pass/Fail — xem Entry #3)</t>
+          <t>Nếu có phần "Sản phẩm liên quan" ở cuối trang, bấm vào một sản phẩm liên quan điều hướng đúng sang trang chi tiết của sản phẩm đó (xác nhận tính năng tồn tại trước khi Pass/Fail, xem Entry #3)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1776,14 +1760,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Xác nhận trên cả 5/5 sản phẩm: không có phần "Sản phẩm liên quan" nào tồn tại trong SUT — theo quyết định ở Entry #3 (`ai-audit-report.md`), đánh N/A thay vì Failed</t>
+          <t>Xác nhận trên cả 5/5 sản phẩm: không có phần "Sản phẩm liên quan" nào tồn tại trong SUT, theo quyết định ở Entry #3 (`ai-audit-report.md`), đánh N/A thay vì Failed</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -1815,17 +1799,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Không thể kiểm thử — cả breadcrumb và sản phẩm liên quan đều không tồn tại trên trang; đây là item về tính năng breadcrumb *bắt buộc* (không có "nếu có" như GUI-030), nên sự vắng mặt hoàn toàn của nó tính là Failed, không phải N/A</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr"/>
+          <t>Không thể kiểm thử: cả breadcrumb và sản phẩm liên quan đều không tồn tại trên trang; đây là item về tính năng breadcrumb *bắt buộc* (không có "nếu có" như GUI-030), nên sự vắng mặt hoàn toàn của nó tính là Failed, không phải N/A</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-004-005-012-023-026-detail-page.png</t>
+        </is>
+      </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
           <t>BUG-IA03-PRODUCTDETAIL-001</t>
@@ -1858,17 +1846,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Không thể kiểm thử — cùng lý do GUI-031, breadcrumb không tồn tại</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr"/>
+          <t>Không thể kiểm thử: cùng lý do GUI-031, breadcrumb không tồn tại</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-004-005-012-023-026-detail-page.png</t>
+        </is>
+      </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
           <t>BUG-IA03-PRODUCTDETAIL-001</t>
@@ -1901,14 +1893,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Không có toast notification nào tồn tại; rà soát navbar ở nhiều trạng thái giỏ hàng khác nhau cũng không thấy badge số lượng. Phản hồi duy nhất là chữ trên chính nút đổi thành "Đã thêm" trong 2 giây — và chỉ xảy ra sau lần bấm **thứ hai** liên tiếp (lần đầu luôn bị bỏ qua im lặng, xem BUG-IA04-PRODUCTDETAIL-001)</t>
+          <t>Không có toast notification nào tồn tại; rà soát navbar ở nhiều trạng thái giỏ hàng khác nhau cũng không thấy badge số lượng. Phản hồi duy nhất là chữ trên chính nút đổi thành "Đã thêm" trong 2 giây, và chỉ xảy ra sau lần bấm **thứ hai** liên tiếp (lần đầu luôn bị bỏ qua im lặng, xem BUG-IA04-PRODUCTDETAIL-001)</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -1948,17 +1940,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Không có toast thực sự để đánh giá thời lượng/khả năng đóng sớm — chỉ có chữ trên nút tự đổi lại sau 2 giây, không có nút đóng</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr"/>
+          <t>Không có toast thực sự để đánh giá thời lượng/khả năng đóng sớm, chỉ có chữ trên nút tự đổi lại sau 2 giây, không có nút đóng</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-038-039-044-046-cart-lost-after-reload.png</t>
+        </is>
+      </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
           <t>BUG-IA04-PRODUCTDETAIL-001</t>
@@ -1991,7 +1987,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2022,7 +2018,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Nếu sản phẩm hết hàng, trang hiển thị rõ trạng thái "Hết hàng" và nút "Thêm vào giỏ hàng" bị disable, không cho bấm (xác nhận SUT có cơ chế tồn kho trước khi Pass/Fail — xem Entry #4)</t>
+          <t>Nếu sản phẩm hết hàng, trang hiển thị rõ trạng thái "Hết hàng" và nút "Thêm vào giỏ hàng" bị disable, không cho bấm (xác nhận SUT có cơ chế tồn kho trước khi Pass/Fail, xem Entry #4)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2030,14 +2026,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Xác nhận qua API `GET /api/products`: không có trường tồn kho/stock nào trong data model của cả 5 sản phẩm — SUT không có cơ chế hết hàng, theo quyết định Entry #4 đánh N/A</t>
+          <t>Xác nhận qua API `GET /api/products`: không có trường tồn kho/stock nào trong data model của cả 5 sản phẩm, SUT không có cơ chế hết hàng, theo quyết định Entry #4 đánh N/A</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
@@ -2069,17 +2065,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Nút không bao giờ chuyển sang trạng thái disable trong bất kỳ tình huống nào (số lượng không hợp lệ, đang xử lý, hết hàng) nên không có style disable để đánh giá — bản thân việc không bao giờ disable là một defect (xem GUI-020)</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr"/>
+          <t>Nút không bao giờ chuyển sang trạng thái disable trong bất kỳ tình huống nào (số lượng không hợp lệ, đang xử lý, hết hàng) nên không có style disable để đánh giá, bản thân việc không bao giờ disable là một defect (xem GUI-020)</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-013-015-017-020-021-cart-qty-zero-accepted.png</t>
+        </is>
+      </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
           <t>BUG-IA02-PRODUCTDETAIL-001</t>
@@ -2112,14 +2112,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Không có bất kỳ lệnh gọi mạng nào cho hành động thêm giỏ hàng (0 network request quan sát được qua tab Network) — do đó không bao giờ có thể xảy ra lỗi mạng/server theo đúng nghĩa để hiển thị thông báo; vấn đề còn nghiêm trọng hơn wording của item: giỏ hàng "thành công" giả tạo vì chưa từng được lưu bền vững ở đâu cả</t>
+          <t>Không có bất kỳ lệnh gọi mạng nào cho hành động thêm giỏ hàng (0 network request quan sát được qua tab Network), do đó không bao giờ có thể xảy ra lỗi mạng/server theo đúng nghĩa để hiển thị thông báo; vấn đề còn nghiêm trọng hơn wording của item: giỏ hàng "thành công" giả tạo vì chưa từng được lưu bền vững ở đâu cả</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2159,17 +2159,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Không có request nào tới server nên không có gì để "chờ" — không có spinner nào tồn tại vì thao tác hoàn toàn đồng bộ ở client, trái với kỳ vọng của FR-06/FR-24 về một thao tác thêm giỏ hàng thực sự</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr"/>
+          <t>Không có request nào tới server nên không có gì để "chờ", không có spinner nào tồn tại vì thao tác hoàn toàn đồng bộ ở client, trái với kỳ vọng của FR-06/FR-24 về một thao tác thêm giỏ hàng thực sự</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-038-039-044-046-cart-lost-after-reload.png</t>
+        </is>
+      </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
           <t>BUG-IA04-PRODUCTDETAIL-001</t>
@@ -2202,14 +2206,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Thêm sản phẩm vào giỏ rồi kiểm tra navbar ở mọi trang — link "Giỏ hàng" không có badge số lượng trong bất kỳ trường hợp nào — vi phạm FR-23</t>
+          <t>Thêm sản phẩm vào giỏ rồi kiểm tra navbar ở mọi trang, link "Giỏ hàng" không có badge số lượng trong bất kỳ trường hợp nào, vi phạm FR-23</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2249,17 +2253,21 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Không có badge/toast để phản ánh (xem GUI-033/040); thêm nữa, thêm cùng sản phẩm 2 lần rồi vào giỏ hàng cho thấy 2 dòng riêng biệt thay vì 1 dòng đã cộng dồn số lượng — vi phạm cả FR-07</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr"/>
+          <t>Không có badge/toast để phản ánh (xem GUI-033/040); thêm nữa, thêm cùng sản phẩm 2 lần rồi vào giỏ hàng cho thấy 2 dòng riêng biệt thay vì 1 dòng đã cộng dồn số lượng, vi phạm cả FR-07</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-068-081-cart-no-badge-duplicate-rows.png</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
           <t>BUG-IA04-PRODUCTDETAIL-001</t>
@@ -2292,14 +2300,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F43" s="3" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Quét toàn bộ `document.styleSheets` xác nhận 0 rule `@media (prefers-color-scheme: dark)` trong toàn bộ CSS — trang dùng màu Tailwind cố định (hardcoded), nên hiển thị giống hệt nhau bất kể chế độ sáng/tối của hệ điều hành; độ tương phản do đó không đổi so với kết quả đã đo ở GUI-010</t>
+          <t>Quét toàn bộ `document.styleSheets` xác nhận 0 rule `@media (prefers-color-scheme: dark)` trong toàn bộ CSS, trang dùng màu Tailwind cố định (hardcoded), nên hiển thị giống hệt nhau bất kể chế độ sáng/tối của hệ điều hành; độ tương phản do đó không đổi so với kết quả đã đo ở GUI-010</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
@@ -2331,7 +2339,7 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2370,14 +2378,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Không thể xảy ra kịch bản này theo đúng nghĩa vì hành động thêm giỏ hàng không hề gọi API (không kiểm tra JWT/session ở bất kỳ đâu) — do đó không có đường xử lý hết phiên nào tồn tại, item không được thỏa mãn dù theo cách nào</t>
+          <t>Không thể xảy ra kịch bản này theo đúng nghĩa vì hành động thêm giỏ hàng không hề gọi API (không kiểm tra JWT/session ở bất kỳ đâu), do đó không có đường xử lý hết phiên nào tồn tại, item không được thỏa mãn dù theo cách nào</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -2417,14 +2425,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Quan sát trực tiếp trên "Bàn phím cơ Keychron Q1", "Tai nghe AirPods Pro 2", "Điện thoại cao cấp của Apple" — toàn bộ dấu tiếng Việt hiển thị đúng, không vỡ font/tofu box (Danh mục thì không có trường nào để kiểm tra dấu — xem GUI-005)</t>
+          <t>Quan sát trực tiếp trên "Bàn phím cơ Keychron Q1", "Tai nghe AirPods Pro 2", "Điện thoại cao cấp của Apple", toàn bộ dấu tiếng Việt hiển thị đúng, không vỡ font/tofu box (Danh mục thì không có trường nào để kiểm tra dấu, xem GUI-005)</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
@@ -2448,7 +2456,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Khi mạng chậm (throttle 3G) lúc bấm "Thêm vào giỏ hàng", không bị treo spinner vô thời hạn — có timeout và thông báo lỗi rõ ràng nếu request quá lâu, thay vì im lặng chờ mãi</t>
+          <t>Khi mạng chậm (throttle 3G) lúc bấm "Thêm vào giỏ hàng", không bị treo spinner vô thời hạn, có timeout và thông báo lỗi rõ ràng nếu request quá lâu, thay vì im lặng chờ mãi</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -2456,17 +2464,21 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="F47" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Không có network request nào cho hành động này (xem GUI-038/039) nên không có gì để throttle/timeout — về mặt kỹ thuật "không treo spinner" là đúng, nhưng chỉ vì tính năng chưa từng thực sự tồn tại, không phải vì được xử lý tốt</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="inlineStr"/>
+          <t>Không có network request nào cho hành động này (xem GUI-038/039) nên không có gì để throttle/timeout, về mặt kỹ thuật "không treo spinner" là đúng, nhưng chỉ vì tính năng chưa từng thực sự tồn tại, không phải vì được xử lý tốt</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-038-039-044-046-cart-lost-after-reload.png</t>
+        </is>
+      </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
           <t>BUG-IA04-PRODUCTDETAIL-001</t>
@@ -2499,14 +2511,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>`document.querySelectorAll('h1')` trả về 2 phần tử: "Danh sách sản phẩm" và "Hiển thị 5 sản phẩm" — dòng thống kê cuối danh sách sản phẩm bị gắn nhầm thẻ `&lt;h1&gt;` thứ hai</t>
+          <t>`document.querySelectorAll('h1')` trả về 2 phần tử: "Danh sách sản phẩm" và "Hiển thị 5 sản phẩm", dòng thống kê cuối danh sách sản phẩm bị gắn nhầm thẻ `&lt;h1&gt;` thứ hai</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2546,7 +2558,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F49" s="3" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2585,14 +2597,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Hiển thị "30,000,000 VND" (chữ VND, dùng dấu phẩy) trên cả 5 sản phẩm, trong khi Product Detail và Giỏ hàng cùng hệ thống hiển thị "30,000,000 đ" — không nhất quán</t>
+          <t>Hiển thị "30,000,000 VND" (chữ VND, dùng dấu phẩy) trên cả 5 sản phẩm, trong khi Product Detail và Giỏ hàng cùng hệ thống hiển thị "30,000,000 đ", không nhất quán</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2632,7 +2644,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F51" s="3" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2663,7 +2675,7 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Mỗi thẻ sản phẩm trong lưới hiển thị đủ Ảnh, Tên, Giá — không thiếu trường nào so với yêu cầu</t>
+          <t>Mỗi thẻ sản phẩm trong lưới hiển thị đủ Ảnh, Tên, Giá, không thiếu trường nào so với yêu cầu</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2671,7 +2683,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F52" s="3" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2710,14 +2722,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F53" s="3" t="inlineStr">
+      <c r="F53" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>`class="w-full h-48 object-cover"` — `object-cover` crop ảnh giữ đúng tỷ lệ, không kéo giãn méo hình</t>
+          <t>`class="w-full h-48 object-cover"`: `object-cover` crop ảnh giữ đúng tỷ lệ, không kéo giãn méo hình</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
@@ -2741,7 +2753,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Tên sản phẩm dài (&gt;60 ký tự) không làm vỡ layout thẻ sản phẩm — có truncate hoặc wrap hợp lý, không tràn ra ngoài khung hoặc đè lên thẻ bên cạnh</t>
+          <t>Tên sản phẩm dài (&gt;60 ký tự) không làm vỡ layout thẻ sản phẩm, có truncate hoặc wrap hợp lý, không tràn ra ngoài khung hoặc đè lên thẻ bên cạnh</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2749,14 +2761,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F54" s="3" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Test bằng cách tạm chèn tên dài 100+ ký tự vào `&lt;h2&gt;` thật qua DOM: class `truncate` (Tailwind: `overflow:hidden; white-space:nowrap; text-overflow:ellipsis`) hoạt động đúng — `cardClientWidth` không đổi (313px), không tràn khung</t>
+          <t>Test bằng cách tạm chèn tên dài 100+ ký tự vào `&lt;h2&gt;` thật qua DOM: class `truncate` (Tailwind: `overflow:hidden; white-space:nowrap; text-overflow:ellipsis`) hoạt động đúng, `cardClientWidth` không đổi (313px), không tràn khung</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
@@ -2788,14 +2800,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F55" s="3" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>`grid grid-cols-1 sm:grid-cols-2 md:grid-cols-3 gap-6` — các thẻ canh đều, khoảng cách nhất quán ở cả 3 breakpoint đã test</t>
+          <t>`grid grid-cols-1 sm:grid-cols-2 md:grid-cols-3 gap-6`: các thẻ canh đều, khoảng cách nhất quán ở cả 3 breakpoint đã test</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -2827,7 +2839,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2866,14 +2878,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F57" s="4" t="inlineStr">
+      <c r="F57" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Đo bằng công thức WCAG relative luminance qua JS: tên (đen/trắng) 21:1 đạt chuẩn, nhưng giá (`text-red-500` rgb(239,68,68)/trắng) chỉ đạt **3.76:1**, dưới ngưỡng 4.5:1 — Product Detail dùng `text-red-600` đậm hơn cho cùng vai trò và đạt 4.83:1</t>
+          <t>Đo bằng công thức WCAG relative luminance qua JS: tên (đen/trắng) 21:1 đạt chuẩn, nhưng giá (`text-red-500` rgb(239,68,68)/trắng) chỉ đạt **3.76:1**, dưới ngưỡng 4.5:1, Product Detail dùng `text-red-600` đậm hơn cho cùng vai trò và đạt 4.83:1</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2905,7 +2917,7 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Layout responsive hợp lý ở cả desktop, tablet và mobile — số cột của lưới sản phẩm tự điều chỉnh, không đè/tràn nội dung</t>
+          <t>Layout responsive hợp lý ở cả desktop, tablet và mobile, số cột của lưới sản phẩm tự điều chỉnh, không đè/tràn nội dung</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2913,14 +2925,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Test ở 1568px (3 cột), và ~625px (giới hạn nhỏ nhất công cụ resize cho phép, tương đương mobile — 1 cột) — không phát hiện chồng lấn/tràn ở cả hai</t>
+          <t>Test ở 1568px (3 cột), và ~625px (giới hạn nhỏ nhất công cụ resize cho phép, tương đương mobile, 1 cột), không phát hiện chồng lấn/tràn ở cả hai</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
@@ -2952,14 +2964,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F59" s="4" t="inlineStr">
+      <c r="F59" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Quan sát nhiều lần tải/reload trang — không có bất kỳ spinner/skeleton nào xuất hiện ở bất kỳ thời điểm nào trong lúc chờ response</t>
+          <t>Quan sát nhiều lần tải/reload trang: không có bất kỳ spinner/skeleton nào xuất hiện ở bất kỳ thời điểm nào trong lúc chờ response</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -2991,7 +3003,7 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>Ô tìm kiếm có placeholder rõ ràng ("Tìm kiếm...") nhưng không dùng placeholder thay thế hoàn toàn cho nhãn — vẫn cần có cách xác định mục đích ô nhập cho screen reader</t>
+          <t>Ô tìm kiếm có placeholder rõ ràng ("Tìm kiếm...") nhưng không dùng placeholder thay thế hoàn toàn cho nhãn, vẫn cần có cách xác định mục đích ô nhập cho screen reader</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2999,14 +3011,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="F60" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Kiểm tra qua Accessibility tree (DevTools): không có `aria-label` hay `&lt;label&gt;` liên kết — khi người dùng gõ, placeholder biến mất và không còn mô tả nào cho screen reader</t>
+          <t>Kiểm tra qua Accessibility tree (DevTools): không có `aria-label` hay `&lt;label&gt;` liên kết, khi người dùng gõ, placeholder biến mất và không còn mô tả nào cho screen reader</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3046,14 +3058,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F61" s="4" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Gõ `&lt;img src=x onerror="window.__xss_fired=true"&gt;` — ảnh vỡ thực sự render trong DOM (không phải văn bản escape), `window.__xss_fired === true` xác nhận script đã thực thi (reflected XSS). Đồng thời phát hiện thêm: request tới `/api/products` trả về lỗi HTTP 500 với thông báo `SQLITE_ERROR` thô do dấu `"` trong payload làm vỡ cú pháp truy vấn phía server — xem BUG-IA02-HOMEPAGE-003 (SQL Injection, phát hiện phụ trong lúc test item này)</t>
+          <t>Gõ `&lt;img src=x onerror="window.__xss_fired=true"&gt;`: ảnh vỡ thực sự render trong DOM (không phải văn bản escape), `window.__xss_fired === true` xác nhận script đã thực thi (reflected XSS). Đồng thời phát hiện thêm: request tới `/api/products` trả về lỗi HTTP 500 với thông báo `SQLITE_ERROR` thô do dấu `"` trong payload làm vỡ cú pháp truy vấn phía server, xem BUG-IA02-HOMEPAGE-003 (SQL Injection, phát hiện phụ trong lúc test item này)</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3093,7 +3105,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F62" s="3" t="inlineStr">
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3132,7 +3144,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr">
+      <c r="F63" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3171,14 +3183,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
+      <c r="F64" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>Cùng nguyên nhân GUI-058 — không có state loading nào trong `fetchProducts`, nút "Tìm" không bao giờ bị disable trong lúc chờ</t>
+          <t>Cùng biểu hiện với GUI-058: không có chỉ báo loading nào xuất hiện, và nút "Tìm" không bao giờ chuyển sang trạng thái disable trong lúc chờ kết quả</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -3218,14 +3230,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F65" s="4" t="inlineStr">
+      <c r="F65" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Cùng phát hiện với GUI-060: không chỉ "làm vỡ layout", ký tự đặc biệt còn (a) thực thi được HTML/JS ở frontend (XSS xác nhận) và (b) làm vỡ câu truy vấn ở backend (lộ lỗi CSDL thô), và khi dùng payload `zzz' OR '1'='1' -- ` thì **bypass hoàn toàn điều kiện tìm kiếm, trả về toàn bộ 5 sản phẩm** dù từ khóa không khớp gì — hành vi này chỉ có thể xảy ra nếu chuỗi nhập vào được nối trực tiếp vào câu SQL phía server, không qua tham số hóa — xác nhận SQL Injection thật (error-based + boolean-based)</t>
+          <t>Cùng phát hiện với GUI-060: không chỉ "làm vỡ layout", ký tự đặc biệt còn (a) thực thi được HTML/JS ở frontend (XSS xác nhận) và (b) làm vỡ câu truy vấn ở backend (lộ lỗi CSDL thô), và khi dùng payload `zzz' OR '1'='1' -- ` thì **bypass hoàn toàn điều kiện tìm kiếm, trả về toàn bộ 5 sản phẩm** dù từ khóa không khớp gì, hành vi này chỉ có thể xảy ra nếu chuỗi nhập vào được nối trực tiếp vào câu SQL phía server, không qua tham số hóa, xác nhận SQL Injection thật (error-based + boolean-based)</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -3265,14 +3277,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F66" s="3" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Test Tab thực tế: ô tìm kiếm → nút "Tìm" (`outline: rgb(0,95,204) auto` focus ring rõ) → link "Xem chi tiết" sản phẩm đầu tiên — đúng thứ tự trên xuống dưới, trái sang phải</t>
+          <t>Test Tab thực tế: ô tìm kiếm → nút "Tìm" (`outline: rgb(0,95,204) auto` focus ring rõ) → link "Xem chi tiết" sản phẩm đầu tiên, đúng thứ tự trên xuống dưới, trái sang phải</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -3304,7 +3316,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F67" s="3" t="inlineStr">
+      <c r="F67" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3343,14 +3355,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="F68" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Đọc DOM `&lt;nav&gt;`: chỉ có "Giỏ hàng", "Chào, Test User", "Thoát" — không có mục "Trang chủ" nào trong nav, và không có active-state class nào thay đổi theo route ở bất kỳ link nào (logo "EShop" nằm ngoài `&lt;nav&gt;`, link về "/" nhưng không style active)</t>
+          <t>Đọc DOM `&lt;nav&gt;`: chỉ có "Giỏ hàng", "Chào, Test User", "Thoát", không có mục "Trang chủ" nào trong nav, và không có active-state class nào thay đổi theo route ở bất kỳ link nào (logo "EShop" nằm ngoài `&lt;nav&gt;`, link về "/" nhưng không style active)</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -3390,14 +3402,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F69" s="4" t="inlineStr">
+      <c r="F69" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Thêm 2 sản phẩm vào giỏ từ trang chủ rồi quan sát navbar: link "Giỏ hàng" không có badge số lượng nào — cùng root cause với BUG-IA04-PRODUCTDETAIL-001 (không có badge/toast ở bất kỳ đâu trong hệ thống)</t>
+          <t>Thêm 2 sản phẩm vào giỏ từ trang chủ rồi quan sát navbar: link "Giỏ hàng" không có badge số lượng nào, cùng root cause với BUG-IA04-PRODUCTDETAIL-001 (không có badge/toast ở bất kỳ đâu trong hệ thống)</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -3437,7 +3449,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F70" s="3" t="inlineStr">
+      <c r="F70" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3476,7 +3488,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F71" s="3" t="inlineStr">
+      <c r="F71" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3515,14 +3527,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F72" s="4" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Tìm "pro" (còn 3 sản phẩm) → vào chi tiết MacBook Pro M3 → bấm Back → trang chủ hiển thị lại **toàn bộ 5 sản phẩm**, ô tìm kiếm trống, dòng "Kết quả tìm kiếm cho: pro" biến mất hoàn toàn — do `useEffect` gọi lại `fetchProducts()` không kèm query mỗi khi component mount lại và `search` không được lưu ở URL</t>
+          <t>Tìm "pro" (còn 3 sản phẩm) → vào chi tiết MacBook Pro M3 → bấm Back → trang chủ hiển thị lại **toàn bộ 5 sản phẩm**, ô tìm kiếm trống, dòng "Kết quả tìm kiếm cho: pro" biến mất hoàn toàn, URL của trang không hề mang từ khóa tìm kiếm, nên khi quay lại, danh sách được tải lại ở trạng thái mặc định</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -3562,7 +3574,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F73" s="3" t="inlineStr">
+      <c r="F73" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3601,7 +3613,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F74" s="3" t="inlineStr">
+      <c r="F74" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3640,7 +3652,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F75" s="4" t="inlineStr">
+      <c r="F75" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -3679,7 +3691,7 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Trang chủ không hiển thị breadcrumb thừa dạng "Trang chủ &gt; Trang chủ" — đúng vì đây là trang gốc, không phải trang con nên breadcrumb theo FR-23 không bắt buộc ở đây</t>
+          <t>Trang chủ không hiển thị breadcrumb thừa dạng "Trang chủ &gt; Trang chủ", đúng vì đây là trang gốc, không phải trang con nên breadcrumb theo FR-23 không bắt buộc ở đây</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
@@ -3687,14 +3699,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F76" s="3" t="inlineStr">
+      <c r="F76" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Xác nhận không có breadcrumb nào trên trang chủ — đúng theo FR-23 (breadcrumb chỉ bắt buộc ở trang con)</t>
+          <t>Xác nhận không có breadcrumb nào trên trang chủ, đúng theo FR-23 (breadcrumb chỉ bắt buộc ở trang con)</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
@@ -3726,14 +3738,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F77" s="4" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Bấm "Thêm vào giỏ" trên thẻ iPhone 15 Pro Max — không có toast, không có badge, không có bất kỳ thay đổi trực quan nào trên trang (khác Product Detail vốn ít nhất đổi chữ nút) — xác nhận sản phẩm có vào giỏ thật (qua SPA navigation tới /cart) nhưng zero phản hồi tại chỗ</t>
+          <t>Bấm "Thêm vào giỏ" trên thẻ iPhone 15 Pro Max, không có toast, không có badge, không có bất kỳ thay đổi trực quan nào trên trang (khác Product Detail vốn ít nhất đổi chữ nút), xác nhận sản phẩm có vào giỏ thật (qua SPA navigation tới /cart) nhưng zero phản hồi tại chỗ</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -3773,7 +3785,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F78" s="4" t="inlineStr">
+      <c r="F78" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -3783,7 +3795,11 @@
           <t>Không có toast nào tồn tại để đánh giá thời lượng/khả năng đóng sớm (hệ quả trực tiếp của GUI-076)</t>
         </is>
       </c>
-      <c r="H78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-068-081-cart-no-badge-duplicate-rows.png</t>
+        </is>
+      </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
           <t>BUG-IA04-PRODUCTDETAIL-001</t>
@@ -3816,14 +3832,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F79" s="4" t="inlineStr">
+      <c r="F79" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>`[...document.querySelectorAll('img')].map(img =&gt; img.getAttribute('alt'))` trả về `["", "", "", "", ""]` cho cả 5 ảnh — thuộc tính `alt` hiện diện nhưng để trống</t>
+          <t>`[...document.querySelectorAll('img')].map(img =&gt; img.getAttribute('alt'))` trả về `["", "", "", "", ""]` cho cả 5 ảnh: thuộc tính `alt` hiện diện nhưng để trống</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -3863,14 +3879,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F80" s="4" t="inlineStr">
+      <c r="F80" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Mô phỏng lỗi mạng thật (patch `XMLHttpRequest` để request `/api/products` luôn fail) rồi tìm kiếm — giao diện **âm thầm hiển thị lại toàn bộ 5 sản phẩm cũ** kèm dòng "Kết quả tìm kiếm cho: ..." như thể thành công, không một thông báo lỗi nào, không log console nào — do khối `catch` trong `fetchProducts` chỉ xử lý khi `err.response.data` là string, lỗi mạng thật không có `err.response` nên bị bỏ qua hoàn toàn</t>
+          <t>Mô phỏng lỗi mạng thật (patch `XMLHttpRequest` để request `/api/products` luôn fail) rồi tìm kiếm, giao diện **âm thầm hiển thị lại toàn bộ 5 sản phẩm cũ** kèm dòng "Kết quả tìm kiếm cho: ..." như thể thành công, không một thông báo lỗi nào, không log console nào, lỗi mạng thật bị nuốt hoàn toàn: không thông báo trên giao diện, không log ra console, dữ liệu cũ vẫn nằm nguyên trên màn hình</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -3902,22 +3918,22 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Khi người dùng tìm kiếm lại (bấm nút Tìm lần thứ 2 trở đi trong cùng phiên), danh sách sản phẩm cũ không biến mất đột ngột thành trắng trơn trong lúc chờ kết quả mới — có trạng thái loading/transition rõ ràng riêng cho hành động tìm kiếm, khác với loading lần đầu tải trang (đã có ở GUI-058)</t>
+          <t>Khi người dùng tìm kiếm lại (bấm nút Tìm lần thứ 2 trở đi trong cùng phiên), danh sách sản phẩm cũ không biến mất đột ngột thành trắng trơn trong lúc chờ kết quả mới, có trạng thái loading/transition rõ ràng riêng cho hành động tìm kiếm, khác với loading lần đầu tải trang (đã có ở GUI-058)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>AI (sửa bởi Human — xem Entry #10 ai-audit-report.md)</t>
-        </is>
-      </c>
-      <c r="F81" s="4" t="inlineStr">
+          <t>AI (sửa bởi Human, xem Entry #10 ai-audit-report.md)</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Cùng root cause GUI-058/063 — không có state loading nào trong `fetchProducts`, dùng chung cho cả tải lần đầu và tìm kiếm lại</t>
+          <t>Cùng biểu hiện với GUI-058/063: không có chỉ báo loading nào, cả khi tải trang lần đầu lẫn khi tìm kiếm lại</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -3957,14 +3973,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F82" s="4" t="inlineStr">
+      <c r="F82" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Bấm "Thêm vào giỏ" 2 lần liên tiếp cho iPhone 15 Pro Max từ trang chủ rồi vào Giỏ hàng — giỏ hiển thị **2 dòng riêng biệt** "iPhone 15 Pro Max, Số lượng: 1" thay vì 1 dòng "Số lượng: 2", tổng tiền 60,000,000 đ thay vì 1 dòng ×2</t>
+          <t>Bấm "Thêm vào giỏ" 2 lần liên tiếp cho iPhone 15 Pro Max từ trang chủ rồi vào Giỏ hàng, giỏ hiển thị **2 dòng riêng biệt** "iPhone 15 Pro Max, Số lượng: 1" thay vì 1 dòng "Số lượng: 2", tổng tiền 60,000,000 đ thay vì 1 dòng ×2</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -3996,7 +4012,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Khi mạng chậm lúc bấm "Thêm vào giỏ" từ trang chủ, không bị treo vô thời hạn — có timeout hoặc thông báo rõ ràng nếu request quá lâu</t>
+          <t>Khi mạng chậm lúc bấm "Thêm vào giỏ" từ trang chủ, không bị treo vô thời hạn, có timeout hoặc thông báo rõ ràng nếu request quá lâu</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -4004,14 +4020,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F83" s="4" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Không có network request nào cho hành động "Thêm vào giỏ" (client-side thuần) nên không có gì để timeout — về mặt kỹ thuật "không treo" là đúng, nhưng chỉ vì tính năng gọi API chưa từng tồn tại, cùng loại phát hiện như GUI-046 (Product Detail)</t>
+          <t>Không có network request nào cho hành động "Thêm vào giỏ" (client-side thuần) nên không có gì để timeout, về mặt kỹ thuật "không treo" là đúng, nhưng chỉ vì tính năng gọi API chưa từng tồn tại, cùng loại phát hiện như GUI-046 (Product Detail)</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -4051,14 +4067,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F84" s="3" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Xác nhận qua thao tác thật: bấm **đúng 1 lần** "Thêm vào giỏ" trên iPhone 15 Pro Max rồi vào Giỏ hàng (SPA navigation) — sản phẩm đã có trong giỏ ngay từ lần bấm đầu, khác với Product Detail vốn cần đúng 2 lần bấm</t>
+          <t>Xác nhận qua thao tác thật: bấm **đúng 1 lần** "Thêm vào giỏ" trên iPhone 15 Pro Max rồi vào Giỏ hàng (SPA navigation), sản phẩm đã có trong giỏ ngay từ lần bấm đầu, khác với Product Detail vốn cần đúng 2 lần bấm</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -4090,14 +4106,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F85" s="3" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Quét `document.styleSheets` xác nhận 0 rule `@media (prefers-color-scheme: dark)` — trang dùng màu Tailwind cố định, hiển thị giống hệt nhau bất kể chế độ sáng/tối hệ điều hành; độ tương phản không đổi so với GUI-056 (giá vẫn có vấn đề contrast riêng, đã ghi nhận ở BUG-IA01-HOMEPAGE-003, không phải do dark mode)</t>
+          <t>Quét `document.styleSheets` xác nhận 0 rule `@media (prefers-color-scheme: dark)`: trang dùng màu Tailwind cố định, hiển thị giống hệt nhau bất kể chế độ sáng/tối hệ điều hành; độ tương phản không đổi so với GUI-056 (giá vẫn có vấn đề contrast riêng, đã ghi nhận ở BUG-IA01-HOMEPAGE-003, không phải do dark mode)</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -4129,7 +4145,7 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F86" s="3" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -4160,7 +4176,7 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Nút "Thêm vào giỏ" trên mỗi thẻ sản phẩm ở trang chủ luôn thêm số lượng mặc định là 1 mà không có ô/chỉ báo nào cho người dùng biết hoặc điều chỉnh số lượng trước khi thêm — cần rõ ràng về số lượng sẽ thêm để tránh hiểu nhầm</t>
+          <t>Nút "Thêm vào giỏ" trên mỗi thẻ sản phẩm ở trang chủ luôn thêm số lượng mặc định là 1 mà không có ô/chỉ báo nào cho người dùng biết hoặc điều chỉnh số lượng trước khi thêm, cần rõ ràng về số lượng sẽ thêm để tránh hiểu nhầm</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
@@ -4168,18 +4184,26 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F87" s="4" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Xác nhận qua DOM và source: card sản phẩm trên trang chủ chỉ có 1 nút "Thêm vào giỏ" (`onClick={() =&gt; addToCart({...p, quantity: 1}, 1)}`), không có ô/hiển thị số lượng nào — khác biệt thiết kế thật với Product Detail (có ô Số lượng theo FR-06), nhưng không vi phạm FR cụ thể nào nên không file bug riêng, chỉ ghi nhận là quan sát UX</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr"/>
-      <c r="I87" s="2" t="inlineStr"/>
+          <t>Xác nhận qua DOM: card sản phẩm trên trang chủ chỉ có đúng 1 nút "Thêm vào giỏ", không có ô nhập hay chỉ báo số lượng nào. Kiểm chứng bằng hành vi: mỗi lần bấm luôn thêm đúng 1 đơn vị vào giỏ, khác biệt thiết kế thật với Product Detail (có ô Số lượng theo FR-06), nhưng không vi phạm FR cụ thể nào nên không file bug riêng, chỉ ghi nhận là quan sát UX</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>checklist/screenshots/GUI-086-home-card-no-quantity.png</t>
+        </is>
+      </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>BUG-IA02-HOMEPAGE-004</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -4207,14 +4231,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F88" s="3" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Dòng thông báo dùng class `mb-4 text-gray-600` (nhỏ hơn, màu xám) trong khi `&lt;h1&gt;` dùng `text-3xl font-bold` — không cùng cỡ chữ theo đúng nghĩa đen của item, nhưng đây là pattern caption phụ chuẩn (cùng bảng màu/font Tailwind của toàn trang), không phải style vỡ/ngẫu hứng. Đánh Passed theo tinh thần thật của item (nhất quán style hệ thống), ghi chú lại vì câu chữ gốc của item hơi quá cụ thể so với ý định — xem Entry #23 ai-audit-report.md</t>
+          <t>Dòng thông báo dùng class `mb-4 text-gray-600` (nhỏ hơn, màu xám) trong khi `&lt;h1&gt;` dùng `text-3xl font-bold`, không cùng cỡ chữ theo đúng nghĩa đen của item, nhưng đây là pattern caption phụ chuẩn (cùng bảng màu/font Tailwind của toàn trang), không phải style vỡ/ngẫu hứng. Đánh Passed theo tinh thần thật của item (nhất quán style hệ thống), ghi chú lại vì câu chữ gốc của item hơi quá cụ thể so với ý định, xem Entry #23 ai-audit-report.md</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr"/>
@@ -4246,14 +4270,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F89" s="3" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Kiểm thử lặp lại nhiều lần kể cả ở các trạng thái lưới bị lỗi/lệch dữ liệu (xem GUI-096): dòng "Hiển thị N sản phẩm" luôn khớp chính xác với `document.querySelectorAll('img').length` thực tế — 2 con số này luôn nhất quán với nhau, dù đôi khi cả 2 cùng sai so với từ khóa đang tìm (root cause riêng, xem BUG-IA04-SEARCHRESULTS-002)</t>
+          <t>Kiểm thử lặp lại nhiều lần kể cả ở các trạng thái lưới bị lỗi/lệch dữ liệu (xem GUI-096): dòng "Hiển thị N sản phẩm" luôn khớp chính xác với `document.querySelectorAll('img').length` thực tế, 2 con số này luôn nhất quán với nhau, dù đôi khi cả 2 cùng sai so với từ khóa đang tìm (root cause riêng, xem BUG-IA04-SEARCHRESULTS-002)</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr"/>
@@ -4285,7 +4309,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F90" s="3" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -4324,14 +4348,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F91" s="4" t="inlineStr">
+      <c r="F91" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Quét toàn bộ `a,button` trên trang ở trạng thái đang xem kết quả: chỉ có "Giỏ hàng", "Chào, Test User", "Thoát", "Tìm", "Xem chi tiết", "Thêm vào giỏ" — không có nút/link "Xóa bộ lọc"/"Xem tất cả" nào</t>
+          <t>Quét toàn bộ `a,button` trên trang ở trạng thái đang xem kết quả: chỉ có "Giỏ hàng", "Chào, Test User", "Thoát", "Tìm", "Xem chi tiết", "Thêm vào giỏ", không có nút/link "Xóa bộ lọc"/"Xem tất cả" nào</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -4371,14 +4395,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F92" s="4" t="inlineStr">
+      <c r="F92" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Sau khi submit tìm kiếm hợp lệ ra đúng 3 kết quả, `location.href` vẫn là `http://localhost:5173/`, `location.search` là chuỗi rỗng — URL không bao giờ phản ánh từ khóa đang tìm. Cùng root cause với BUG-IA03-HOMEPAGE-002</t>
+          <t>Sau khi submit tìm kiếm hợp lệ ra đúng 3 kết quả, `location.href` vẫn là `http://localhost:5173/`, `location.search` là chuỗi rỗng, URL không bao giờ phản ánh từ khóa đang tìm. Cùng root cause với BUG-IA03-HOMEPAGE-002</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -4418,14 +4442,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F93" s="4" t="inlineStr">
+      <c r="F93" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Sau khi bấm "Tìm" (submit thật), `document.activeElement` vẫn là nút "Tìm" — không có cơ chế nào chủ động chuyển focus tới vùng kết quả mới</t>
+          <t>Sau khi bấm "Tìm" (submit thật), `document.activeElement` vẫn là nút "Tìm", không có cơ chế nào chủ động chuyển focus tới vùng kết quả mới</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -4457,22 +4481,22 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Nếu có phân trang hoặc infinite scroll cho kết quả tìm kiếm (xác nhận tính năng tồn tại trước khi Pass/Fail — theo quy ước N/A đã dùng ở GUI-019/030), việc chuyển trang kết quả vẫn giữ nguyên từ khóa đang tìm kiếm, không bị mất/reset về danh sách đầy đủ</t>
+          <t>Nếu có phân trang hoặc infinite scroll cho kết quả tìm kiếm (xác nhận tính năng tồn tại trước khi Pass/Fail, theo quy ước N/A đã dùng ở GUI-019/030), việc chuyển trang kết quả vẫn giữ nguyên từ khóa đang tìm kiếm, không bị mất/reset về danh sách đầy đủ</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>AI (sửa bởi Human — xem Entry #15 ai-audit-report.md)</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
+          <t>AI (sửa bởi Human, xem Entry #15 ai-audit-report.md)</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Quét toàn bộ `document.body.innerHTML` không tìm thấy bất kỳ từ khóa nào liên quan phân trang ("pagination", "phân trang", "trang sau", "xem thêm"...) — SUT chỉ có 5 sản phẩm nên không có tính năng phân trang nào tồn tại để kiểm thử</t>
+          <t>Quét toàn bộ `document.body.innerHTML` không tìm thấy bất kỳ từ khóa nào liên quan phân trang ("pagination", "phân trang", "trang sau", "xem thêm"...), SUT chỉ có 5 sản phẩm nên không có tính năng phân trang nào tồn tại để kiểm thử</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr"/>
@@ -4504,14 +4528,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F95" s="4" t="inlineStr">
+      <c r="F95" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Điều hướng trực tiếp tới `http://localhost:5173/?search=pro` — trang tải lên với ô tìm kiếm trống, không có dòng "Kết quả tìm kiếm cho", hiển thị toàn bộ 5 sản phẩm mặc định, hoàn toàn bỏ qua query param `search`. Cùng root cause với BUG-IA03-HOMEPAGE-002</t>
+          <t>Điều hướng trực tiếp tới `http://localhost:5173/?search=pro`: trang tải lên với ô tìm kiếm trống, không có dòng "Kết quả tìm kiếm cho", hiển thị toàn bộ 5 sản phẩm mặc định, hoàn toàn bỏ qua query param `search`. Cùng root cause với BUG-IA03-HOMEPAGE-002</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -4551,14 +4575,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F96" s="4" t="inlineStr">
+      <c r="F96" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>`document.querySelectorAll('[aria-live]').length === 0` ở mọi trạng thái đã kiểm thử (có kết quả, không kết quả) — không có `aria-live` nào tồn tại trên toàn trang</t>
+          <t>`document.querySelectorAll('[aria-live]').length === 0` ở mọi trạng thái đã kiểm thử (có kết quả, không kết quả), không có `aria-live` nào tồn tại trên toàn trang</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -4598,14 +4622,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F97" s="4" t="inlineStr">
+      <c r="F97" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>**Phát hiện quan trọng**: gõ "macbook" vào ô tìm kiếm mà KHÔNG bấm "Tìm" — dòng "Kết quả tìm kiếm cho: macbook" cập nhật ngay theo từng ký tự gõ, nhưng lưới sản phẩm vẫn giữ nguyên toàn bộ 5 sản phẩm cũ (đúng ra chỉ 1: MacBook Pro M3) — xác nhận qua DOM `input.value === 'macbook'` nhưng `imgCount === 5`. Lặp lại nhiều lần với từ khóa khác nhau: hành vi không nhất quán giữa các lần thao tác giống hệt — đôi khi lưới tự cập nhật live theo ký tự gõ, đôi khi chỉ cập nhật khi bấm "Tìm"/Enter, trong khi dòng chú thích luôn cập nhật ngay lập tức bất kể lưới đã đồng bộ hay chưa. Trạng thái lệch có thể tồn tại không giới hạn thời gian tới khi người dùng chủ động submit</t>
+          <t>**Phát hiện quan trọng**: gõ "macbook" vào ô tìm kiếm mà KHÔNG bấm "Tìm", dòng "Kết quả tìm kiếm cho: macbook" cập nhật ngay theo từng ký tự gõ, nhưng lưới sản phẩm vẫn giữ nguyên toàn bộ 5 sản phẩm cũ (đúng ra chỉ 1: MacBook Pro M3), xác nhận qua DOM `input.value === 'macbook'` nhưng `imgCount === 5`. Lặp lại nhiều lần với từ khóa khác nhau: hành vi không nhất quán giữa các lần thao tác giống hệt, đôi khi lưới tự cập nhật live theo ký tự gõ, đôi khi chỉ cập nhật khi bấm "Tìm"/Enter, trong khi dòng chú thích luôn cập nhật ngay lập tức bất kể lưới đã đồng bộ hay chưa. Trạng thái lệch có thể tồn tại không giới hạn thời gian tới khi người dùng chủ động submit</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -4645,14 +4669,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F98" s="4" t="inlineStr">
+      <c r="F98" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Từ trạng thái đang xem đúng 3 kết quả "pro", patch XHR để `/api/products` luôn fail, rồi submit tìm kiếm mới "iphone" — dòng chú thích cập nhật thành "iphone" nhưng lưới vẫn giữ nguyên 3 sản phẩm cũ của "pro", không một chữ lỗi nào xuất hiện (`/lỗi|error|thất bại/i` không khớp bất kỳ đâu trong `body.innerText`). Cùng root cause, ngữ cảnh mới so với BUG-IA04-HOMEPAGE-003</t>
+          <t>Từ trạng thái đang xem đúng 3 kết quả "pro", patch XHR để `/api/products` luôn fail, rồi submit tìm kiếm mới "iphone", dòng chú thích cập nhật thành "iphone" nhưng lưới vẫn giữ nguyên 3 sản phẩm cũ của "pro", không một chữ lỗi nào xuất hiện: rà toàn bộ văn bản hiển thị trên trang không tìm thấy bất kỳ từ nào thuộc nhóm "lỗi", "error", "thất bại". Cùng root cause, ngữ cảnh mới so với BUG-IA04-HOMEPAGE-003</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -4692,14 +4716,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F99" s="4" t="inlineStr">
+      <c r="F99" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Gọi trực tiếp API để cô lập khỏi các bất ổn khác của giao diện: `GET /api/products?search=iphone` → 1 kết quả; `GET /api/products?search=%20iphone%20` (có khoảng trắng đầu/cuối) → 0 kết quả. Xác nhận lại qua UI: submit " iphone " ra đúng 0 sản phẩm dù "iphone" một mình cho 1 kết quả — backend không trim khoảng trắng</t>
+          <t>Gọi trực tiếp API để cô lập khỏi các bất ổn khác của giao diện: `GET /api/products?search=iphone` → 1 kết quả; `GET /api/products?search=%20iphone%20` (có khoảng trắng đầu/cuối) → 0 kết quả. Xác nhận lại qua UI: submit " iphone " ra đúng 0 sản phẩm dù "iphone" một mình cho 1 kết quả, backend không trim khoảng trắng</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -4739,14 +4763,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F100" s="3" t="inlineStr">
+      <c r="F100" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Quét `document.styleSheets` xác nhận 0 rule `@media (prefers-color-scheme: dark)` — trang dùng màu Tailwind cố định, hiển thị giống hệt nhau bất kể chế độ sáng/tối hệ điều hành, cùng kết luận như GUI-042/084</t>
+          <t>Quét `document.styleSheets` xác nhận 0 rule `@media (prefers-color-scheme: dark)`: trang dùng màu Tailwind cố định, hiển thị giống hệt nhau bất kể chế độ sáng/tối hệ điều hành, cùng kết luận như GUI-042/084</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr"/>
@@ -4778,14 +4802,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F101" s="4" t="inlineStr">
+      <c r="F101" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Tìm kiếm "zzznotfound" (submit thật, xác nhận 0 kết quả hợp lệ) — toàn bộ phần dưới dòng "Kết quả tìm kiếm cho" là khoảng trắng hoàn toàn: `document.querySelectorAll('img').length === 0`, `svg.length === 0`, không có message nào — vi phạm trực tiếp FR-05/FR-24</t>
+          <t>Tìm kiếm "zzznotfound" (submit thật, xác nhận 0 kết quả hợp lệ), toàn bộ phần dưới dòng "Kết quả tìm kiếm cho" là khoảng trắng hoàn toàn: `document.querySelectorAll('img').length === 0`, `svg.length === 0`, không có message nào, vi phạm trực tiếp FR-05/FR-24</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -4817,7 +4841,7 @@
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái trống responsive tốt trên mobile — icon/hình minh họa và thông điệp không bị tràn, vỡ layout, hoặc bị cắt ở màn hình hẹp</t>
+          <t>Trạng thái trống responsive tốt trên mobile, icon/hình minh họa và thông điệp không bị tràn, vỡ layout, hoặc bị cắt ở màn hình hẹp</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
@@ -4825,14 +4849,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F102" s="4" t="inlineStr">
+      <c r="F102" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Hệ quả trực tiếp của GUI-100: vì không có icon/message nào tồn tại ở bất kỳ độ rộng nào, không có gì để đánh giá là "responsive tốt" — theo đúng nguyên tắc đã áp dụng cho breadcrumb (GUI-023→024/025/031/032), tính năng bắt buộc (FR-24) vắng mặt hoàn toàn tính là Failed cho mọi item phụ thuộc, không phải N/A</t>
+          <t>Hệ quả trực tiếp của GUI-100: vì không có icon/message nào tồn tại ở bất kỳ độ rộng nào, không có gì để đánh giá là "responsive tốt", theo đúng nguyên tắc đã áp dụng cho breadcrumb (GUI-023→024/025/031/032), tính năng bắt buộc (FR-24) vắng mặt hoàn toàn tính là Failed cho mọi item phụ thuộc, không phải N/A</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -4872,14 +4896,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F103" s="3" t="inlineStr">
+      <c r="F103" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Sau khi submit "zzznotfound" ra 0 kết quả, `document.querySelector('input').value === 'zzznotfound'` — ô tìm kiếm giữ đúng nguyên văn từ khóa</t>
+          <t>Sau khi submit "zzznotfound" ra 0 kết quả, `document.querySelector('input').value === 'zzznotfound'`, ô tìm kiếm giữ đúng nguyên văn từ khóa</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr"/>
@@ -4903,22 +4927,22 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Thông điệp trạng thái trống gợi ý cụ thể ít nhất một hành động tiếp theo — hoặc một nút/link rõ ràng để xem lại toàn bộ sản phẩm, hoặc gợi ý kiểm tra lại chính tả từ khóa — không chỉ nói chung chung "không có sản phẩm" rồi để người dùng tự loay hoay</t>
+          <t>Thông điệp trạng thái trống gợi ý cụ thể ít nhất một hành động tiếp theo, hoặc một nút/link rõ ràng để xem lại toàn bộ sản phẩm, hoặc gợi ý kiểm tra lại chính tả từ khóa, không chỉ nói chung chung "không có sản phẩm" rồi để người dùng tự loay hoay</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>AI (sửa bởi Human — xem Entry #19 ai-audit-report.md)</t>
-        </is>
-      </c>
-      <c r="F104" s="4" t="inlineStr">
+          <t>AI (sửa bởi Human, xem Entry #19 ai-audit-report.md)</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Hệ quả trực tiếp của GUI-100: không tồn tại bất kỳ message nào (thân thiện hay chung chung) — nên chắc chắn không có gợi ý hành động nào</t>
+          <t>Hệ quả trực tiếp của GUI-100: không tồn tại bất kỳ message nào (thân thiện hay chung chung), nên chắc chắn không có gợi ý hành động nào</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -4958,14 +4982,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F105" s="4" t="inlineStr">
+      <c r="F105" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Quét `a,button` ở trạng thái trống: chỉ còn navbar ("Giỏ hàng", "Chào, Test User", "Thoát") và nút "Tìm" — không có link/nút "Xem tất cả sản phẩm" nào, đúng là dead-end nếu không tự xóa tay ô tìm kiếm</t>
+          <t>Quét `a,button` ở trạng thái trống: chỉ còn navbar ("Giỏ hàng", "Chào, Test User", "Thoát") và nút "Tìm", không có link/nút "Xem tất cả sản phẩm" nào, đúng là dead-end nếu không tự xóa tay ô tìm kiếm</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -5005,7 +5029,7 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F106" s="4" t="inlineStr">
+      <c r="F106" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -5044,7 +5068,7 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Khi tìm kiếm với từ khóa không khớp sản phẩm nào, hệ thống thực sự hiển thị trạng thái "không tìm thấy" — không lặng lẽ hiển thị lại toàn bộ danh sách sản phẩm cũ như thể tìm kiếm thành công, cùng loại lỗi với BUG-IA04-HOMEPAGE-003 đã ghi nhận</t>
+          <t>Khi tìm kiếm với từ khóa không khớp sản phẩm nào, hệ thống thực sự hiển thị trạng thái "không tìm thấy", không lặng lẽ hiển thị lại toàn bộ danh sách sản phẩm cũ như thể tìm kiếm thành công, cùng loại lỗi với BUG-IA04-HOMEPAGE-003 đã ghi nhận</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
@@ -5052,14 +5076,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F107" s="3" t="inlineStr">
+      <c r="F107" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Khi tìm kiếm được submit đúng cách (gõ + bấm "Tìm") với từ khóa chắc chắn không khớp, lưới sản phẩm thực sự trả về 0 kết quả (`imgCount === 0`), không fallback về danh sách cũ — khác với lo ngại ban đầu, hành vi "giữ dữ liệu cũ" (GUI-096/097) chỉ xảy ra ở trạng thái transient trước khi submit hoặc khi có lỗi mạng thật, không xảy ra với một tìm kiếm 0-kết-quả hợp lệ đã hoàn tất</t>
+          <t>Khi tìm kiếm được submit đúng cách (gõ + bấm "Tìm") với từ khóa chắc chắn không khớp, lưới sản phẩm thực sự trả về 0 kết quả (`imgCount === 0`), không fallback về danh sách cũ, khác với lo ngại ban đầu, hành vi "giữ dữ liệu cũ" (GUI-096/097) chỉ xảy ra ở trạng thái transient trước khi submit hoặc khi có lỗi mạng thật, không xảy ra với một tìm kiếm 0-kết-quả hợp lệ đã hoàn tất</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr"/>
@@ -5083,22 +5107,22 @@
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Nếu một truy vấn tìm kiếm gây ra lỗi thật ở backend (không phải trường hợp 0 kết quả hợp lệ), giao diện không được âm thầm hiển thị lẫn thành trạng thái "không tìm thấy sản phẩm" thân thiện — phải phân biệt được lỗi hệ thống thật với 0 kết quả tìm kiếm thật, tránh che giấu lỗi dưới vỏ bọc UX thân thiện</t>
+          <t>Nếu một truy vấn tìm kiếm gây ra lỗi thật ở backend (không phải trường hợp 0 kết quả hợp lệ), giao diện không được âm thầm hiển thị lẫn thành trạng thái "không tìm thấy sản phẩm" thân thiện, phải phân biệt được lỗi hệ thống thật với 0 kết quả tìm kiếm thật, tránh che giấu lỗi dưới vỏ bọc UX thân thiện</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>AI (sửa bởi Human — xem Entry #21 ai-audit-report.md)</t>
-        </is>
-      </c>
-      <c r="F108" s="3" t="inlineStr">
+          <t>AI (sửa bởi Human, xem Entry #21 ai-audit-report.md)</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Test với payload `test'quote` (dấu nháy đơn lẻ) — xác nhận qua API trực tiếp đây là lỗi thật (`HTTP 500`, `SQLITE_ERROR: near "quote": syntax error`). Qua UI, lỗi này KHÔNG bị hiển thị lẫn thành "không tìm thấy" — trang hiển thị nguyên văn khối "Database Error / SQLITE_ERROR..." trong khung màu đỏ, khác hẳn (và tệ hơn) so với trạng thái trống thật (hoàn toàn không có gì). 2 trạng thái về mặt kỹ thuật CÓ thể phân biệt được, nhưng chỉ vì lỗi thật bị rò rỉ thô ra UI (đã ghi nhận ở BUG-IA02-HOMEPAGE-002/003), không phải do có chủ đích thiết kế phân biệt 2 trạng thái — nếu rò rỉ lỗi thô được vá lại bằng một thông báo lỗi chung chung "thân thiện" mà KHÔNG đồng thời vá GUI-100 (trạng thái trống trơn), nguy cơ nhầm lẫn đúng như item lo ngại sẽ xuất hiện trở lại</t>
+          <t>Test với payload `test'quote` (dấu nháy đơn lẻ), xác nhận qua API trực tiếp đây là lỗi thật (`HTTP 500`, `SQLITE_ERROR: near "quote": syntax error`). Qua UI, lỗi này KHÔNG bị hiển thị lẫn thành "không tìm thấy", trang hiển thị nguyên văn khối "Database Error / SQLITE_ERROR..." trong khung màu đỏ, khác hẳn (và tệ hơn) so với trạng thái trống thật (hoàn toàn không có gì). 2 trạng thái về mặt kỹ thuật CÓ thể phân biệt được, nhưng chỉ vì lỗi thật bị rò rỉ thô ra UI (đã ghi nhận ở BUG-IA02-HOMEPAGE-002/003), không phải do có chủ đích thiết kế phân biệt 2 trạng thái, nếu rò rỉ lỗi thô được vá lại bằng một thông báo lỗi chung chung "thân thiện" mà KHÔNG đồng thời vá GUI-100 (trạng thái trống trơn), nguy cơ nhầm lẫn đúng như item lo ngại sẽ xuất hiện trở lại</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr"/>
@@ -5130,14 +5154,14 @@
           <t>AI</t>
         </is>
       </c>
-      <c r="F109" s="4" t="inlineStr">
+      <c r="F109" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>`document.querySelectorAll('[aria-live]').length === 0` ở trạng thái trống — không có `aria-live` nào tồn tại (cùng phát hiện với GUI-095 ở Search Results, một root cause chung toàn ứng dụng)</t>
+          <t>`document.querySelectorAll('[aria-live]').length === 0` ở trạng thái trống: không có `aria-live` nào tồn tại (cùng phát hiện với GUI-095 ở Search Results, một root cause chung toàn ứng dụng)</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
@@ -5177,14 +5201,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F110" s="3" t="inlineStr">
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Submit "khôngtồntại" (có đủ dấu tiếng Việt) — dấu hiển thị đúng cả trong ô tìm kiếm lẫn dòng "Kết quả tìm kiếm cho", không vỡ font/tofu box, và trả về đúng 0 sản phẩm (không bị hiểu nhầm thành thành công như trường hợp GUI-096/097)</t>
+          <t>Submit "khôngtồntại" (có đủ dấu tiếng Việt), dấu hiển thị đúng cả trong ô tìm kiếm lẫn dòng "Kết quả tìm kiếm cho", không vỡ font/tofu box, và trả về đúng 0 sản phẩm (không bị hiểu nhầm thành thành công như trường hợp GUI-096/097)</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr"/>
@@ -5216,14 +5240,14 @@
           <t>Human</t>
         </is>
       </c>
-      <c r="F111" s="4" t="inlineStr">
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Hệ quả trực tiếp của GUI-100: không có icon/thông điệp nào tồn tại ở bất kỳ chế độ màu nào để đánh giá độ tương phản — khác với GUI-099 (Search Results) nơi các phần tử văn bản thực sự tồn tại và có thể đo contrast, ở đây không có gì để đo</t>
+          <t>Hệ quả trực tiếp của GUI-100: không có icon/thông điệp nào tồn tại ở bất kỳ chế độ màu nào để đánh giá độ tương phản, khác với GUI-099 (Search Results) nơi các phần tử văn bản thực sự tồn tại và có thể đo contrast, ở đây không có gì để đo</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -5241,4 +5265,241 @@
   <autoFilter ref="A1:I111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>HW03 Task 1 - GUI Checklist test summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Ha Bao Ngoc - 23127300</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SUT</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>EShop (eshop-sut @ 85af3ba) - http://localhost:5173/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Screens tested</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Product Detail, Home Page, Search Results, Empty Search State</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>IA aspect</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>Designed</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>IA01 - General UI standards</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>34</v>
+      </c>
+      <c r="C8" t="n">
+        <v>34</v>
+      </c>
+      <c r="D8" t="n">
+        <v>24</v>
+      </c>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>IA02 - Forms</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>27</v>
+      </c>
+      <c r="C9" t="n">
+        <v>27</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12</v>
+      </c>
+      <c r="E9" t="n">
+        <v>14</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IA03 - Navigation</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>24</v>
+      </c>
+      <c r="C10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7</v>
+      </c>
+      <c r="E10" t="n">
+        <v>15</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>IA04 - Feedback / state</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25</v>
+      </c>
+      <c r="C11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="n">
+        <v>20</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Items from AI first pass</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Items added by human review</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Distinct bugs filed</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>24</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>